<commit_message>
xyz company report structure completed
</commit_message>
<xml_diff>
--- a/Trial Balance.xlsx
+++ b/Trial Balance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shivam Chaturvedi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\Drishti Web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED618D39-67D9-41CB-B7E9-96764BD24C33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7FADDB4-121E-4A65-A947-17F71077E522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1883,15 +1883,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E246"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1908,7 +1909,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1925,7 +1926,7 @@
         <v>-1365970</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1942,7 +1943,7 @@
         <v>-868680</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>-2888560445.96</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
@@ -1976,7 +1977,7 @@
         <v>2371971.39</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
@@ -1993,7 +1994,7 @@
         <v>7941080.54</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -2010,7 +2011,7 @@
         <v>-38668.9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
@@ -2027,7 +2028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>0</v>
       </c>
@@ -2044,7 +2045,7 @@
         <v>1284522.43</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>0</v>
       </c>
@@ -2061,7 +2062,7 @@
         <v>-2000000000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
@@ -2078,7 +2079,7 @@
         <v>-400000000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
@@ -2095,7 +2096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>0</v>
       </c>
@@ -2112,7 +2113,7 @@
         <v>-247462601.78999999</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>0</v>
       </c>
@@ -2129,7 +2130,7 @@
         <v>-238523.49</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>0</v>
       </c>
@@ -2146,7 +2147,7 @@
         <v>-1940219</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>0</v>
       </c>
@@ -2163,7 +2164,7 @@
         <v>-2662538</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>0</v>
       </c>
@@ -2180,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>0</v>
       </c>
@@ -2197,7 +2198,7 @@
         <v>-265968343.41</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>0</v>
       </c>
@@ -2214,7 +2215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>0</v>
       </c>
@@ -2231,7 +2232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>0</v>
       </c>
@@ -2248,7 +2249,7 @@
         <v>-23799281.010000002</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>0</v>
       </c>
@@ -2265,7 +2266,7 @@
         <v>-53207755.670000002</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>0</v>
       </c>
@@ -2282,7 +2283,7 @@
         <v>-6382962</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>0</v>
       </c>
@@ -2299,7 +2300,7 @@
         <v>-7927826.0199999996</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>0</v>
       </c>
@@ -2316,7 +2317,7 @@
         <v>-167825540.69999999</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>0</v>
       </c>
@@ -2333,7 +2334,7 @@
         <v>-78704.78</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>0</v>
       </c>
@@ -2350,7 +2351,7 @@
         <v>179382.89</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>0</v>
       </c>
@@ -2367,7 +2368,7 @@
         <v>-48270629.700000003</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>0</v>
       </c>
@@ -2384,7 +2385,7 @@
         <v>-311807</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>0</v>
       </c>
@@ -2401,7 +2402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>0</v>
       </c>
@@ -2418,7 +2419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>0</v>
       </c>
@@ -2435,7 +2436,7 @@
         <v>-6369417.54</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>0</v>
       </c>
@@ -2452,7 +2453,7 @@
         <v>-2295777</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>0</v>
       </c>
@@ -2469,7 +2470,7 @@
         <v>-1443331.5</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>0</v>
       </c>
@@ -2486,7 +2487,7 @@
         <v>-6010925.9900000002</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>0</v>
       </c>
@@ -2503,7 +2504,7 @@
         <v>-604915.06000000006</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>0</v>
       </c>
@@ -2520,7 +2521,7 @@
         <v>-1218102.76</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>0</v>
       </c>
@@ -2537,7 +2538,7 @@
         <v>-995290.17</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>0</v>
       </c>
@@ -2554,7 +2555,7 @@
         <v>-21113</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>0</v>
       </c>
@@ -2571,7 +2572,7 @@
         <v>-64627</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>0</v>
       </c>
@@ -2588,7 +2589,7 @@
         <v>-627704</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>0</v>
       </c>
@@ -2605,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>0</v>
       </c>
@@ -2622,7 +2623,7 @@
         <v>-288873</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>0</v>
       </c>
@@ -2639,7 +2640,7 @@
         <v>-31400</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>0</v>
       </c>
@@ -2656,7 +2657,7 @@
         <v>-1683162</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>0</v>
       </c>
@@ -2673,7 +2674,7 @@
         <v>-104173676.48</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>0</v>
       </c>
@@ -2690,7 +2691,7 @@
         <v>93599471</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>0</v>
       </c>
@@ -2707,7 +2708,7 @@
         <v>1479119263.8</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>0</v>
       </c>
@@ -2724,7 +2725,7 @@
         <v>-23521985.120000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>0</v>
       </c>
@@ -2741,7 +2742,7 @@
         <v>3385169564.52</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>0</v>
       </c>
@@ -2758,7 +2759,7 @@
         <v>-98387307.799999997</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>0</v>
       </c>
@@ -2775,7 +2776,7 @@
         <v>19595727</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>0</v>
       </c>
@@ -2792,7 +2793,7 @@
         <v>-1127057.1200000001</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>0</v>
       </c>
@@ -2809,7 +2810,7 @@
         <v>16903685.710000001</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>0</v>
       </c>
@@ -2826,7 +2827,7 @@
         <v>-1509878.12</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>0</v>
       </c>
@@ -2843,7 +2844,7 @@
         <v>20587570.109999999</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>0</v>
       </c>
@@ -2860,7 +2861,7 @@
         <v>-594660.1</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>0</v>
       </c>
@@ -2877,7 +2878,7 @@
         <v>133494755.59</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>0</v>
       </c>
@@ -2894,7 +2895,7 @@
         <v>-3890620.15</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>0</v>
       </c>
@@ -2911,7 +2912,7 @@
         <v>4679369.24</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>0</v>
       </c>
@@ -2928,7 +2929,7 @@
         <v>-314295.84999999998</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>0</v>
       </c>
@@ -2945,7 +2946,7 @@
         <v>324389641</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>0</v>
       </c>
@@ -2962,7 +2963,7 @@
         <v>-9297332.9299999997</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>0</v>
       </c>
@@ -2979,7 +2980,7 @@
         <v>60.24</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>0</v>
       </c>
@@ -2996,7 +2997,7 @@
         <v>11010528.060000001</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>0</v>
       </c>
@@ -3013,7 +3014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>0</v>
       </c>
@@ -3030,7 +3031,7 @@
         <v>-41060</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>0</v>
       </c>
@@ -3047,7 +3048,7 @@
         <v>41000</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>0</v>
       </c>
@@ -3064,7 +3065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>0</v>
       </c>
@@ -3081,7 +3082,7 @@
         <v>27413904</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>0</v>
       </c>
@@ -3098,7 +3099,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>0</v>
       </c>
@@ -3115,7 +3116,7 @@
         <v>95917.28</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>0</v>
       </c>
@@ -3132,7 +3133,7 @@
         <v>32146506.07</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>0</v>
       </c>
@@ -3149,7 +3150,7 @@
         <v>2090466.14</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>0</v>
       </c>
@@ -3166,7 +3167,7 @@
         <v>1514975.19</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>0</v>
       </c>
@@ -3183,7 +3184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>0</v>
       </c>
@@ -3200,7 +3201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>0</v>
       </c>
@@ -3217,7 +3218,7 @@
         <v>5470168.6399999997</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>0</v>
       </c>
@@ -3234,7 +3235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>0</v>
       </c>
@@ -3251,7 +3252,7 @@
         <v>39908783.710000001</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>0</v>
       </c>
@@ -3268,7 +3269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>0</v>
       </c>
@@ -3285,7 +3286,7 @@
         <v>44942032.479999997</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>0</v>
       </c>
@@ -3302,7 +3303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>0</v>
       </c>
@@ -3319,7 +3320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>0</v>
       </c>
@@ -3336,7 +3337,7 @@
         <v>633961.30000000005</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>0</v>
       </c>
@@ -3353,7 +3354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>0</v>
       </c>
@@ -3370,7 +3371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>0</v>
       </c>
@@ -3387,7 +3388,7 @@
         <v>-191373.5</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>0</v>
       </c>
@@ -3404,7 +3405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>0</v>
       </c>
@@ -3421,7 +3422,7 @@
         <v>475424.48</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>0</v>
       </c>
@@ -3438,7 +3439,7 @@
         <v>1194993284.8699999</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>0</v>
       </c>
@@ -3455,7 +3456,7 @@
         <v>-1196902487.3299999</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>0</v>
       </c>
@@ -3472,7 +3473,7 @@
         <v>5669741007.0799999</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>0</v>
       </c>
@@ -3489,7 +3490,7 @@
         <v>-5667521755.0799999</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>0</v>
       </c>
@@ -3506,7 +3507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>0</v>
       </c>
@@ -3523,7 +3524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>0</v>
       </c>
@@ -3540,7 +3541,7 @@
         <v>5036678</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>0</v>
       </c>
@@ -3557,7 +3558,7 @@
         <v>35799</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>0</v>
       </c>
@@ -3574,7 +3575,7 @@
         <v>1281187.08</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>0</v>
       </c>
@@ -3591,7 +3592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>0</v>
       </c>
@@ -3608,7 +3609,7 @@
         <v>-16738.64</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>0</v>
       </c>
@@ -3625,7 +3626,7 @@
         <v>-16738.64</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>0</v>
       </c>
@@ -3642,7 +3643,7 @@
         <v>-11013.8</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>0</v>
       </c>
@@ -3659,7 +3660,7 @@
         <v>212112768.58000001</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>0</v>
       </c>
@@ -3676,7 +3677,7 @@
         <v>87084777</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>0</v>
       </c>
@@ -3693,7 +3694,7 @@
         <v>212112768.58000001</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>0</v>
       </c>
@@ -3710,7 +3711,7 @@
         <v>24208.97</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>0</v>
       </c>
@@ -3727,7 +3728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" s="2" t="s">
         <v>0</v>
       </c>
@@ -3744,7 +3745,7 @@
         <v>1497682</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>0</v>
       </c>
@@ -3761,7 +3762,7 @@
         <v>1538643.27</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
         <v>0</v>
       </c>
@@ -3778,7 +3779,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>0</v>
       </c>
@@ -3795,7 +3796,7 @@
         <v>6901653.5</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
         <v>0</v>
       </c>
@@ -3812,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
         <v>0</v>
       </c>
@@ -3829,7 +3830,7 @@
         <v>1424896.13</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>0</v>
       </c>
@@ -3846,7 +3847,7 @@
         <v>1230728.44</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>0</v>
       </c>
@@ -3863,7 +3864,7 @@
         <v>-2896800</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>0</v>
       </c>
@@ -3880,7 +3881,7 @@
         <v>-36004816.200000003</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>0</v>
       </c>
@@ -3897,7 +3898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
         <v>0</v>
       </c>
@@ -3914,7 +3915,7 @@
         <v>-4811525</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>0</v>
       </c>
@@ -3931,7 +3932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
         <v>0</v>
       </c>
@@ -3948,7 +3949,7 @@
         <v>-1375000</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
         <v>0</v>
       </c>
@@ -3965,7 +3966,7 @@
         <v>-69165987.239999995</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" s="2" t="s">
         <v>0</v>
       </c>
@@ -3982,7 +3983,7 @@
         <v>4811525</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
         <v>0</v>
       </c>
@@ -3999,7 +4000,7 @@
         <v>-118301.89</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
         <v>0</v>
       </c>
@@ -4016,7 +4017,7 @@
         <v>-226317.04</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" s="2" t="s">
         <v>0</v>
       </c>
@@ -4033,7 +4034,7 @@
         <v>-1538643.27</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
         <v>0</v>
       </c>
@@ -4050,7 +4051,7 @@
         <v>-250440</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" s="2" t="s">
         <v>0</v>
       </c>
@@ -4067,7 +4068,7 @@
         <v>-67940.179999999993</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
         <v>0</v>
       </c>
@@ -4084,7 +4085,7 @@
         <v>-59812</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
         <v>0</v>
       </c>
@@ -4101,7 +4102,7 @@
         <v>-4891456.13</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
         <v>0</v>
       </c>
@@ -4118,7 +4119,7 @@
         <v>-90892.479999999996</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" s="2" t="s">
         <v>0</v>
       </c>
@@ -4135,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
         <v>0</v>
       </c>
@@ -4152,7 +4153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
         <v>0</v>
       </c>
@@ -4169,7 +4170,7 @@
         <v>-0.08</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
         <v>0</v>
       </c>
@@ -4186,7 +4187,7 @@
         <v>234308.82</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
         <v>0</v>
       </c>
@@ -4203,7 +4204,7 @@
         <v>10000.299999999999</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
         <v>0</v>
       </c>
@@ -4220,7 +4221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
         <v>0</v>
       </c>
@@ -4237,7 +4238,7 @@
         <v>34055264.18</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
         <v>0</v>
       </c>
@@ -4254,7 +4255,7 @@
         <v>72442537.900000006</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
         <v>0</v>
       </c>
@@ -4271,7 +4272,7 @@
         <v>43648143.68</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
         <v>0</v>
       </c>
@@ -4288,7 +4289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
         <v>0</v>
       </c>
@@ -4305,7 +4306,7 @@
         <v>3966283.86</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
         <v>0</v>
       </c>
@@ -4322,7 +4323,7 @@
         <v>177795</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
         <v>0</v>
       </c>
@@ -4339,7 +4340,7 @@
         <v>727168</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
         <v>0</v>
       </c>
@@ -4356,7 +4357,7 @@
         <v>-76405643.700000003</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
         <v>0</v>
       </c>
@@ -4373,7 +4374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
         <v>0</v>
       </c>
@@ -4390,7 +4391,7 @@
         <v>1072575.3600000001</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
         <v>0</v>
       </c>
@@ -4407,7 +4408,7 @@
         <v>-2669.66</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" s="2" t="s">
         <v>0</v>
       </c>
@@ -4424,7 +4425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
         <v>0</v>
       </c>
@@ -4441,7 +4442,7 @@
         <v>10988214.35</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
         <v>0</v>
       </c>
@@ -4458,7 +4459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
         <v>0</v>
       </c>
@@ -4475,7 +4476,7 @@
         <v>-38423397.710000001</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
         <v>0</v>
       </c>
@@ -4492,7 +4493,7 @@
         <v>352846.7</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
         <v>0</v>
       </c>
@@ -4509,7 +4510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
         <v>0</v>
       </c>
@@ -4526,7 +4527,7 @@
         <v>3015834.67</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
         <v>0</v>
       </c>
@@ -4543,7 +4544,7 @@
         <v>23295</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
         <v>0</v>
       </c>
@@ -4560,7 +4561,7 @@
         <v>9562593.3800000008</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
         <v>0</v>
       </c>
@@ -4577,7 +4578,7 @@
         <v>62292</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
         <v>0</v>
       </c>
@@ -4594,7 +4595,7 @@
         <v>579629</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
         <v>0</v>
       </c>
@@ -4611,7 +4612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
         <v>0</v>
       </c>
@@ -4628,7 +4629,7 @@
         <v>2632.26</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
         <v>0</v>
       </c>
@@ -4645,7 +4646,7 @@
         <v>-1178846</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
         <v>0</v>
       </c>
@@ -4662,7 +4663,7 @@
         <v>1240563.73</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
         <v>0</v>
       </c>
@@ -4679,7 +4680,7 @@
         <v>-888759</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
         <v>0</v>
       </c>
@@ -4696,7 +4697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
         <v>0</v>
       </c>
@@ -4713,7 +4714,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
         <v>0</v>
       </c>
@@ -4730,7 +4731,7 @@
         <v>1534987.98</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
         <v>0</v>
       </c>
@@ -4747,7 +4748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169" s="2" t="s">
         <v>0</v>
       </c>
@@ -4764,7 +4765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170" s="2" t="s">
         <v>0</v>
       </c>
@@ -4781,7 +4782,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171" s="2" t="s">
         <v>0</v>
       </c>
@@ -4798,7 +4799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
         <v>0</v>
       </c>
@@ -4815,7 +4816,7 @@
         <v>273238</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
         <v>0</v>
       </c>
@@ -4832,7 +4833,7 @@
         <v>5013308</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" s="2" t="s">
         <v>0</v>
       </c>
@@ -4849,7 +4850,7 @@
         <v>10135.67</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" s="2" t="s">
         <v>0</v>
       </c>
@@ -4866,7 +4867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" s="2" t="s">
         <v>0</v>
       </c>
@@ -4883,7 +4884,7 @@
         <v>50094.559999999998</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
         <v>0</v>
       </c>
@@ -4900,7 +4901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" s="2" t="s">
         <v>0</v>
       </c>
@@ -4917,7 +4918,7 @@
         <v>1192</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" s="2" t="s">
         <v>0</v>
       </c>
@@ -4934,7 +4935,7 @@
         <v>69159839.489999995</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" s="2" t="s">
         <v>0</v>
       </c>
@@ -4951,7 +4952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" s="2" t="s">
         <v>0</v>
       </c>
@@ -4968,7 +4969,7 @@
         <v>2007199</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" s="2" t="s">
         <v>0</v>
       </c>
@@ -4985,7 +4986,7 @@
         <v>47620</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
         <v>0</v>
       </c>
@@ -5002,7 +5003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
         <v>0</v>
       </c>
@@ -5019,7 +5020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
         <v>0</v>
       </c>
@@ -5036,7 +5037,7 @@
         <v>22880378.75</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
         <v>0</v>
       </c>
@@ -5053,7 +5054,7 @@
         <v>95748628.150000006</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
         <v>0</v>
       </c>
@@ -5070,7 +5071,7 @@
         <v>1127057.1200000001</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
         <v>0</v>
       </c>
@@ -5087,7 +5088,7 @@
         <v>1467688.55</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" s="2" t="s">
         <v>0</v>
       </c>
@@ -5104,7 +5105,7 @@
         <v>594660.1</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
         <v>0</v>
       </c>
@@ -5121,7 +5122,7 @@
         <v>3890620.15</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" s="2" t="s">
         <v>0</v>
       </c>
@@ -5138,7 +5139,7 @@
         <v>314295.84999999998</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192" s="2" t="s">
         <v>0</v>
       </c>
@@ -5155,7 +5156,7 @@
         <v>3467334.25</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" s="2" t="s">
         <v>0</v>
       </c>
@@ -5172,7 +5173,7 @@
         <v>9522573.5500000007</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" s="2" t="s">
         <v>0</v>
       </c>
@@ -5189,7 +5190,7 @@
         <v>2027753.38</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" s="2" t="s">
         <v>0</v>
       </c>
@@ -5206,7 +5207,7 @@
         <v>-1570775.47</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" s="2" t="s">
         <v>0</v>
       </c>
@@ -5223,7 +5224,7 @@
         <v>12173006.960000001</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" s="2" t="s">
         <v>0</v>
       </c>
@@ -5240,7 +5241,7 @@
         <v>3914159</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" s="2" t="s">
         <v>0</v>
       </c>
@@ -5257,7 +5258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" s="2" t="s">
         <v>0</v>
       </c>
@@ -5274,7 +5275,7 @@
         <v>643551.84</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" s="2" t="s">
         <v>0</v>
       </c>
@@ -5291,7 +5292,7 @@
         <v>61500</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" s="2" t="s">
         <v>0</v>
       </c>
@@ -5308,7 +5309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" s="2" t="s">
         <v>0</v>
       </c>
@@ -5325,7 +5326,7 @@
         <v>1011893.11</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" s="2" t="s">
         <v>0</v>
       </c>
@@ -5342,7 +5343,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" s="2" t="s">
         <v>0</v>
       </c>
@@ -5359,7 +5360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" s="2" t="s">
         <v>0</v>
       </c>
@@ -5376,7 +5377,7 @@
         <v>6665</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
         <v>0</v>
       </c>
@@ -5393,7 +5394,7 @@
         <v>27691.040000000001</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" s="2" t="s">
         <v>0</v>
       </c>
@@ -5410,7 +5411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" s="2" t="s">
         <v>0</v>
       </c>
@@ -5427,7 +5428,7 @@
         <v>11098.82</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
         <v>0</v>
       </c>
@@ -5444,7 +5445,7 @@
         <v>2941967.12</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
         <v>0</v>
       </c>
@@ -5461,7 +5462,7 @@
         <v>555235.06000000006</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
         <v>0</v>
       </c>
@@ -5478,7 +5479,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
         <v>0</v>
       </c>
@@ -5495,7 +5496,7 @@
         <v>8675890.5999999996</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
         <v>0</v>
       </c>
@@ -5512,7 +5513,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
         <v>0</v>
       </c>
@@ -5529,7 +5530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A215" s="2" t="s">
         <v>0</v>
       </c>
@@ -5546,7 +5547,7 @@
         <v>1105604.24</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
         <v>0</v>
       </c>
@@ -5563,7 +5564,7 @@
         <v>-547.41999999999996</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
         <v>0</v>
       </c>
@@ -5580,7 +5581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A218" s="2" t="s">
         <v>0</v>
       </c>
@@ -5597,7 +5598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A219" s="2" t="s">
         <v>0</v>
       </c>
@@ -5614,7 +5615,7 @@
         <v>512193</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220" s="2" t="s">
         <v>0</v>
       </c>
@@ -5631,7 +5632,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221" s="2" t="s">
         <v>0</v>
       </c>
@@ -5648,7 +5649,7 @@
         <v>330709.64</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222" s="2" t="s">
         <v>0</v>
       </c>
@@ -5665,7 +5666,7 @@
         <v>2022522.17</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223" s="2" t="s">
         <v>0</v>
       </c>
@@ -5682,7 +5683,7 @@
         <v>1201187.3</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" s="2" t="s">
         <v>0</v>
       </c>
@@ -5699,7 +5700,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A225" s="2" t="s">
         <v>0</v>
       </c>
@@ -5716,7 +5717,7 @@
         <v>216090</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A226" s="2" t="s">
         <v>0</v>
       </c>
@@ -5733,7 +5734,7 @@
         <v>221276</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A227" s="2" t="s">
         <v>0</v>
       </c>
@@ -5750,7 +5751,7 @@
         <v>240246.6</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A228" s="2" t="s">
         <v>0</v>
       </c>
@@ -5767,7 +5768,7 @@
         <v>651224.57999999996</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A229" s="2" t="s">
         <v>0</v>
       </c>
@@ -5784,7 +5785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A230" s="2" t="s">
         <v>0</v>
       </c>
@@ -5801,7 +5802,7 @@
         <v>27726.13</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A231" s="2" t="s">
         <v>0</v>
       </c>
@@ -5818,7 +5819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A232" s="2" t="s">
         <v>0</v>
       </c>
@@ -5835,7 +5836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" s="2" t="s">
         <v>0</v>
       </c>
@@ -5852,7 +5853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" s="2" t="s">
         <v>0</v>
       </c>
@@ -5869,7 +5870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" s="2" t="s">
         <v>0</v>
       </c>
@@ -5886,7 +5887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" s="2" t="s">
         <v>0</v>
       </c>
@@ -5903,7 +5904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" s="2" t="s">
         <v>0</v>
       </c>
@@ -5920,7 +5921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" s="2" t="s">
         <v>0</v>
       </c>
@@ -5937,7 +5938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" s="2" t="s">
         <v>0</v>
       </c>
@@ -5954,7 +5955,7 @@
         <v>-1435975.91</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" s="2" t="s">
         <v>0</v>
       </c>
@@ -5971,7 +5972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A241" s="2" t="s">
         <v>0</v>
       </c>
@@ -5988,7 +5989,7 @@
         <v>-1266811.1000000001</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A242" s="2" t="s">
         <v>0</v>
       </c>
@@ -6005,7 +6006,7 @@
         <v>-4175105.67</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A243" s="2" t="s">
         <v>0</v>
       </c>
@@ -6022,7 +6023,7 @@
         <v>227800</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A244" s="2" t="s">
         <v>0</v>
       </c>
@@ -6039,7 +6040,7 @@
         <v>-164579766</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A245" s="2" t="s">
         <v>0</v>
       </c>
@@ -6056,7 +6057,7 @@
         <v>164351966</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A246" s="2" t="s">
         <v>0</v>
       </c>

</xml_diff>